<commit_message>
Deskripsi singkat perubahan yang kamu lakukan
</commit_message>
<xml_diff>
--- a/outputs/3. Digital Security IT Sample Register (Final).xlsx
+++ b/outputs/3. Digital Security IT Sample Register (Final).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,85 +489,40 @@
           <t>Risk Priority (post-mitigation)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Schema Alignment Log</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Risk ID (Reasoning)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Risk Description (Reasoning)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Project Stage (Reasoning)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Project Category (Reasoning)</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Risk Owner (Reasoning)</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Likelihood (Reasoning)</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Impact (Reasoning)</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Mitigating Action (Reasoning)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>R-UNK</t>
+          <t>ICT-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Identity and Access Management (IAM) systems compromised. Systems are susceptible to intrusion from external sources due to web applications supported by out of date operating systems.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Operation</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Uaa Lead</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monitor and evaluate.</t>
+          <t>Implement automated IAM systems and Multiform Authentication where required. Complete Update of new Application Architecture. Data encryption at rest and in transit implemented for all systems. ISO 27001 based Framework and associated relevant controls implemented.</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
         <v>7</v>
@@ -581,78 +536,33 @@
         <v>3</v>
       </c>
       <c r="K2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
+          <t>Med</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>R-UNK</t>
+          <t>ICT-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Backup and recovery services are not documented and untested. Critical Systems are supported by out of date infrastructure and operating systems, resulting in database corruptions.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Operation</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -662,96 +572,51 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Monitor and evaluate.</t>
+          <t>Implement automated IAM systems and Multiform Authentication where required. Complete Update of new Application Architecture. Data encryption at rest and in transit implemented for all systems. ISO 27001 based Framework and associated relevant controls implemented.</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H3" t="n">
         <v>7</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>R-UNK</t>
+          <t>ICT-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Unspecified</t>
+          <t>Critical Systems are supported by out of date infrastructure and operating systems, resulting in numerous outages and untreatable cyber security intrusions. Current infrastructure is not architected for high availability. Lack of Disaster Recovery facilities that will meet Recovery Time and Point Objective requirements</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Operation</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Cybersecurity</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -761,74 +626,29 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Monitor and evaluate.</t>
+          <t>Document and Test Backup and Recovery services. Migrate systems to new Infrastructure. ISO 27001 based Framework and associated relevant controls implemented.</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H4" t="n">
         <v>7</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Med</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Tidak ada alasan.</t>
+          <t>High</t>
         </is>
       </c>
     </row>

</xml_diff>